<commit_message>
chore: fully update tracker for P6-S01/S02 — all columns, doc strategy, dashboard
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v4.xlsx
+++ b/CortexKitchen_Progress_Tracker_v4.xlsx
@@ -1042,7 +1042,7 @@
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="77" t="inlineStr">
         <is>
-          <t>Last completed: P6-00c — drop Diff 1, v3 reseed, stale_assumptions fix (2026-06-26)</t>
+          <t>Last completed: P6-S02 — connectors table + async job queue (2026-06-27)</t>
         </is>
       </c>
       <c r="B4" s="44" t="inlineStr">
@@ -1078,7 +1078,7 @@
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="76" t="inlineStr">
         <is>
-          <t>Stable: main + dev in sync (P6-00a/b/c merged to main 2026-06-27); next: P6-S01</t>
+          <t>Stable: main + dev in sync (P6-S01/S02 merged to dev 2026-06-27); next: P6-S03 (swiggy-sync-orders)</t>
         </is>
       </c>
       <c r="B5" s="49" t="inlineStr">
@@ -13321,12 +13321,12 @@
       </c>
       <c r="H9" s="44" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md (new), docs/ARCHITECTURE.md, CLAUDE.md, docs/DECISIONS.md (D-019)</t>
+          <t>docs/ARCHITECTURE.md (connector layer section), docs/DECISIONS.md (D-019), docs/DATA_MODEL.md, CLAUDE.md (new), docs/SWIGGY_INTEGRATION.md</t>
         </is>
       </c>
       <c r="I9" s="45" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J9" s="46" t="inlineStr">
@@ -13339,14 +13339,18 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L9" s="43" t="inlineStr"/>
+      <c r="L9" s="43" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
       <c r="M9" s="43" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="N9" s="47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" s="44" t="inlineStr">
         <is>
@@ -13355,7 +13359,7 @@
       </c>
       <c r="P9" s="44" t="inlineStr">
         <is>
-          <t>is_available() True/False; call_tool() 401 re-auth + 5xx retry; get_addresses returns data end-to-end</t>
+          <t>13/13 pass — test_swiggy_client.py (7): is_available, 401 no-retry, 500 retry x2, success data, never raises, success=false; test_connector_repository.py (6): upsert create, upsert idempotent, get none, error_count increment, error clear on success, list_active filter</t>
         </is>
       </c>
     </row>
@@ -13397,12 +13401,12 @@
       </c>
       <c r="H10" s="49" t="inlineStr">
         <is>
-          <t>docs/DATA_MODEL.md (connectors table), docs/DATA_SOURCES.md (new), docs/APIS.md (job status endpoint)</t>
+          <t>docs/DATA_MODEL.md (connectors table, orders/reservations/feedback new cols), docs/ARCHITECTURE.md, docs/DECISIONS.md (D-019)</t>
         </is>
       </c>
       <c r="I10" s="45" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J10" s="46" t="inlineStr">
@@ -13415,14 +13419,18 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L10" s="48" t="inlineStr"/>
+      <c r="L10" s="48" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
       <c r="M10" s="48" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="N10" s="50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O10" s="49" t="inlineStr">
         <is>
@@ -13431,7 +13439,7 @@
       </c>
       <c r="P10" s="49" t="inlineStr">
         <is>
-          <t>Migration smoke test; token encryption round-trip; async run returns job_id immediately; status endpoint polls correctly</t>
+          <t>Migration smoke test (alembic upgrade head verified live on DB); connectors table + all new cols confirmed via psycopg2; swiggy_delivery enum value present</t>
         </is>
       </c>
     </row>
@@ -16178,7 +16186,7 @@
       </c>
       <c r="D4" s="72" t="inlineStr">
         <is>
-          <t>New</t>
+          <t>Updated (status + signatures)</t>
         </is>
       </c>
     </row>
@@ -16266,7 +16274,7 @@
       </c>
       <c r="D8" s="73" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Updated (P6-S01/S02 done)</t>
         </is>
       </c>
     </row>
@@ -16332,7 +16340,7 @@
       </c>
       <c r="D11" s="73" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Updated (P6-S02 done)</t>
         </is>
       </c>
     </row>
@@ -16354,7 +16362,7 @@
       </c>
       <c r="D12" s="73" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Updated (D-019 added P6-S01)</t>
         </is>
       </c>
     </row>
@@ -16442,7 +16450,7 @@
       </c>
       <c r="D16" s="73" t="inlineStr">
         <is>
-          <t>Update</t>
+          <t>Created (P6-S01 done)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: add P6-S01/S02 to Phase Tracker, update Git Practices notes, fix header
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v4.xlsx
+++ b/CortexKitchen_Progress_Tracker_v4.xlsx
@@ -7989,7 +7989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q71"/>
+  <dimension ref="A1:Q73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8014,7 +8014,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>CortexKitchen — Phase Tracker (P0 through P6-00c complete)</t>
+          <t>CortexKitchen — Phase Tracker (P0 through P6-S02 complete)</t>
         </is>
       </c>
     </row>
@@ -12864,7 +12864,172 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="8" customHeight="1"/>
+    <row r="72" ht="8" customHeight="1">
+      <c r="A72" s="87" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B72" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" s="88" t="inlineStr">
+        <is>
+          <t>P6-S01</t>
+        </is>
+      </c>
+      <c r="D72" s="88" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="E72" s="88" t="inlineStr">
+        <is>
+          <t>BaseConnector + SwiggyMCPClient</t>
+        </is>
+      </c>
+      <c r="F72" s="88" t="inlineStr">
+        <is>
+          <t>BaseConnector ABC (sync/enrich), SwiggyMCPClient (JSON-RPC 2.0, httpx, graceful degradation — never raises), SwiggyConnector skeleton, enrichers/ + executor/ package stubs, CLAUDE.md at root, swiggy_access_token + swiggy_address_id in settings</t>
+        </is>
+      </c>
+      <c r="G72" s="88" t="inlineStr">
+        <is>
+          <t>feature/swiggy-base-connector</t>
+        </is>
+      </c>
+      <c r="H72" s="84" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I72" s="51" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J72" s="87" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K72" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="L72" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="M72" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="N72" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="O72" s="88" t="inlineStr">
+        <is>
+          <t>P6-00c</t>
+        </is>
+      </c>
+      <c r="P72" s="88" t="inlineStr">
+        <is>
+          <t>7 tests: is_available True/False; call_tool returns None on 401, 500 (x2 retry verified), success data dict, never raises on Exception, returns None on success=false</t>
+        </is>
+      </c>
+      <c r="Q72" s="88" t="inlineStr">
+        <is>
+          <t>Merged to dev 2026-06-27. PR #80. CLAUDE.md created. Migration verified live on DB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="87" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B73" s="87" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" s="88" t="inlineStr">
+        <is>
+          <t>P6-S02</t>
+        </is>
+      </c>
+      <c r="D73" s="88" t="inlineStr">
+        <is>
+          <t>Infra</t>
+        </is>
+      </c>
+      <c r="E73" s="88" t="inlineStr">
+        <is>
+          <t>connectors table + async job queue</t>
+        </is>
+      </c>
+      <c r="F73" s="88" t="inlineStr">
+        <is>
+          <t>Alembic migration b3e1f2a9c5d7: connectors table (11 cols, uq org+type), orders.source/channel/external_order_id, reservations.source/external_booking_id, feedback delivery timing cols, swiggy_delivery enum value. ConnectorRepository (upsert, token, sync status). Redis async job queue (24h TTL, uuid4 IDs, no external library).</t>
+        </is>
+      </c>
+      <c r="G73" s="88" t="inlineStr">
+        <is>
+          <t>feature/swiggy-base-connector</t>
+        </is>
+      </c>
+      <c r="H73" s="84" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I73" s="51" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J73" s="87" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K73" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="L73" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="M73" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="N73" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="O73" s="88" t="inlineStr">
+        <is>
+          <t>P6-S01</t>
+        </is>
+      </c>
+      <c r="P73" s="88" t="inlineStr">
+        <is>
+          <t>6 tests: upsert creates, upsert idempotent (1 row), get returns None, error_count increments, error clears on success, list_active filter. Migration smoke: alembic upgrade head + psycopg2 verify all cols + enum.</t>
+        </is>
+      </c>
+      <c r="Q73" s="88" t="inlineStr">
+        <is>
+          <t>Merged to dev 2026-06-27. PR #80. Migration verified live on Docker Postgres.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A40:Q40"/>
@@ -16619,7 +16784,7 @@
       </c>
       <c r="D4" s="44" t="inlineStr">
         <is>
-          <t>Phase 3 already synced</t>
+          <t>Phase 6 on dev (P6-S01/S02 merged). main has P5 + P6-00 series. Next main sync: end of Phase 6.</t>
         </is>
       </c>
       <c r="E4" s="2" t="n"/>
@@ -16663,7 +16828,7 @@
       </c>
       <c r="D5" s="49" t="inlineStr">
         <is>
-          <t>Current working base</t>
+          <t>Current working base — Phase 6 active (P6-S01/S02 complete, P6-S03 next)</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>

</xml_diff>

<commit_message>
chore: update tracker for P6-S03 — all 5 sheets (Phase 6, Phase Tracker, Doc Strategy, Dashboard, Git Practices)
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v4.xlsx
+++ b/CortexKitchen_Progress_Tracker_v4.xlsx
@@ -1042,7 +1042,7 @@
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="77" t="inlineStr">
         <is>
-          <t>Last completed: P6-S02 — connectors table + async job queue (2026-06-27)</t>
+          <t>Last completed: P6-S03 — SwiggyOrderSyncService, get_food_orders → orders table (2026-06-27)</t>
         </is>
       </c>
       <c r="B4" s="44" t="inlineStr">
@@ -1078,7 +1078,7 @@
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="76" t="inlineStr">
         <is>
-          <t>Stable: main + dev in sync (P6-S01/S02 merged to dev 2026-06-27); next: P6-S03 (swiggy-sync-orders)</t>
+          <t>Stable: main + dev in sync through P6-S03; next: P6-S04 (swiggy-sync-reservations)</t>
         </is>
       </c>
       <c r="B5" s="49" t="inlineStr">
@@ -7989,7 +7989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q73"/>
+  <dimension ref="A1:Q74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13027,6 +13027,89 @@
       <c r="Q73" s="88" t="inlineStr">
         <is>
           <t>Merged to dev 2026-06-27. PR #80. Migration verified live on Docker Postgres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="87" t="inlineStr">
+        <is>
+          <t>Phase 6</t>
+        </is>
+      </c>
+      <c r="B74" s="87" t="n">
+        <v>3</v>
+      </c>
+      <c r="C74" s="88" t="inlineStr">
+        <is>
+          <t>P6-S03</t>
+        </is>
+      </c>
+      <c r="D74" s="88" t="inlineStr">
+        <is>
+          <t>Integrations</t>
+        </is>
+      </c>
+      <c r="E74" s="88" t="inlineStr">
+        <is>
+          <t>SwiggyOrderSyncService — get_food_orders → orders table</t>
+        </is>
+      </c>
+      <c r="F74" s="88" t="inlineStr">
+        <is>
+          <t>SwiggyOrderSyncService.sync(address_id): fetches up to 20 Swiggy delivery orders, creates one Order row per item (source=swiggy, channel=delivery, is_delivery=True, external_order_id={orderId}_{idx}). _get_or_create_menu_item: case-insensitive name match; placeholder (is_available=False) if no match. Idempotent. SwiggyConnector.sync() implemented: reads SWIGGY_ADDRESS_ID, sets connector status syncing→success/error. BaseConnector updated: db: Session added to __init__.</t>
+        </is>
+      </c>
+      <c r="G74" s="88" t="inlineStr">
+        <is>
+          <t>feature/swiggy-sync-orders</t>
+        </is>
+      </c>
+      <c r="H74" s="84" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="I74" s="51" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="J74" s="87" t="inlineStr">
+        <is>
+          <t>Anoushka</t>
+        </is>
+      </c>
+      <c r="K74" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="L74" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="M74" s="87" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="N74" s="87" t="n">
+        <v>1</v>
+      </c>
+      <c r="O74" s="88" t="inlineStr">
+        <is>
+          <t>P6-S02</t>
+        </is>
+      </c>
+      <c r="P74" s="88" t="inlineStr">
+        <is>
+          <t>8/8 pass: correct count, Order fields, placeholder MenuItem, reuse existing MenuItem, idempotency, None graceful, empty list, ext_id format</t>
+        </is>
+      </c>
+      <c r="Q74" s="88" t="inlineStr">
+        <is>
+          <t>Merged to dev 2026-06-27. Mock-first (no Swiggy token needed). Live integration test pending token.</t>
         </is>
       </c>
     </row>
@@ -13669,12 +13752,12 @@
       </c>
       <c r="H13" s="44" t="inlineStr">
         <is>
-          <t>docs/DATA_SOURCES.md (Swiggy orders), docs/DATA_MODEL.md (source+channel cols), docs/AGENTS.md (demand_forecast updated)</t>
+          <t>docs/SWIGGY_INTEGRATION.md (P6-S03 ✅, status header updated)</t>
         </is>
       </c>
       <c r="I13" s="45" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J13" s="51" t="inlineStr">
@@ -13687,14 +13770,18 @@
           <t>Anoushka</t>
         </is>
       </c>
-      <c r="L13" s="43" t="inlineStr"/>
+      <c r="L13" s="43" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
       <c r="M13" s="43" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="N13" s="47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13" s="44" t="inlineStr">
         <is>
@@ -13703,7 +13790,7 @@
       </c>
       <c r="P13" s="44" t="inlineStr">
         <is>
-          <t>Sync idempotency (run twice = no duplicates); ForecastService channel filter test; orders table has source=swiggy rows after sync</t>
+          <t>8/8 pass — correct count, correct Order fields (source/channel/is_delivery), placeholder MenuItem creation (is_available=False, category=swiggy_import), reuse existing MenuItem by name, idempotency on duplicate sync, None call_tool graceful, empty order list, external_order_id format SW-001_0/SW-001_1</t>
         </is>
       </c>
     </row>
@@ -16346,12 +16433,12 @@
       </c>
       <c r="C4" s="49" t="inlineStr">
         <is>
-          <t>P6-D01 — NEW</t>
+          <t>P6-D01 — updated P6-S01/S02/S03</t>
         </is>
       </c>
       <c r="D4" s="72" t="inlineStr">
         <is>
-          <t>Updated (status + signatures)</t>
+          <t>Updated (P6-S03 status ✅)</t>
         </is>
       </c>
     </row>
@@ -16828,7 +16915,7 @@
       </c>
       <c r="D5" s="49" t="inlineStr">
         <is>
-          <t>Current working base — Phase 6 active (P6-S01/S02 complete, P6-S03 next)</t>
+          <t>Current working base — Phase 6 active (P6-S01/S02/S03 complete, P6-S04 next)</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>

</xml_diff>

<commit_message>
feat(P6-S04/D02): remove phase1_sync, update all docs to 11-node graph
- Remove phase1_sync barrier node from graph.py (was a no-op workaround)
- Wire reservation, complaint_intelligence, inventory directly to menu_intelligence
  (LangGraph native fan-in: menu fires once when all 3 predecessors complete)
- Update all 20+ MD files and HTML deep-dive to reflect 11-node graph:
  - 12-node → 11-node everywhere
  - Replace phase1_sync section with Native Fan-In explanation
  - Fix graph topology diagrams and node tables
  - apps/api/README: Phase 6 in progress, Phase 6 additions section, new env vars
  - apps/web/README, infra/README: Phase 6 in progress, circuit breaker in Redis
  - HTML: Phase1 Sync section replaced with Native LangGraph Fan-In
  - Tradeoff #10 updated from phase1_sync overhead to chatbot org_id gap
- Mark P6-S04 Completed (100%) in Phase Tracker sheet
- P6-D02 already Completed in Phase 6 sheet
</commit_message>
<xml_diff>
--- a/CortexKitchen_Progress_Tracker_v4.xlsx
+++ b/CortexKitchen_Progress_Tracker_v4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Phase Tracker" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Phase 6" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Doc Strategy" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Git Practices" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Tracker" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 6" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doc Strategy" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Git Practices" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1042,7 +1042,7 @@
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="77" t="inlineStr">
         <is>
-          <t>Last completed: P6-S03 — SwiggyOrderSyncService, get_food_orders → orders table (2026-06-27)</t>
+          <t>Last completed: P6-S04 — Agent Intelligence Bundle + docs overhaul (phase1_sync removed, all docs updated) (2026-06-29)</t>
         </is>
       </c>
       <c r="B4" s="44" t="inlineStr">
@@ -1078,7 +1078,7 @@
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="76" t="inlineStr">
         <is>
-          <t>Stable: dev through P6-S03; P6-S04 (agent-intelligence) IN PROGRESS → next: P6-S05 (Dineout sync, token pending)</t>
+          <t>Stable: dev through P6-S04; all docs updated to reflect 11-node graph; next: P6-S05 (Dineout sync, token pending) or P6-S07 (CompetitorEnricher)</t>
         </is>
       </c>
       <c r="B5" s="49" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="B6" s="44" t="inlineStr">
         <is>
-          <t>feature/swiggy-base-connector</t>
+          <t>feature/swiggy-market-intel-enrichers</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
@@ -1507,11 +1507,11 @@
       </c>
       <c r="B16" s="66" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="C16" s="79" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="D16" s="49" t="inlineStr">
         <is>
@@ -13149,7 +13149,7 @@
       </c>
       <c r="H75" s="84" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="I75" s="51" t="inlineStr">
@@ -13174,7 +13174,7 @@
       </c>
       <c r="M75" s="87" t="inlineStr"/>
       <c r="N75" s="87" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O75" s="88" t="inlineStr">
         <is>
@@ -13916,7 +13916,7 @@
       </c>
       <c r="I14" s="45" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J14" s="51" t="inlineStr">
@@ -13940,7 +13940,7 @@
         </is>
       </c>
       <c r="N14" s="43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O14" s="44" t="inlineStr">
         <is>
@@ -15981,7 +15981,7 @@
       </c>
       <c r="I53" s="45" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="J53" s="51" t="inlineStr">
@@ -16001,7 +16001,7 @@
         </is>
       </c>
       <c r="N53" s="50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O53" s="49" t="inlineStr">
         <is>

</xml_diff>